<commit_message>
Adiciona módulo de avisos de vencimento
</commit_message>
<xml_diff>
--- a/outputs/exemplo/clientes_exemplo.xlsx
+++ b/outputs/exemplo/clientes_exemplo.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atendimentos" sheetId="1" r:id="Rc79b7a9669a648e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atendimentos" sheetId="1" r:id="R5b155e6c6f6344c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobrancas" sheetId="2" r:id="Rf09b959e3ece44c5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -437,4 +438,75 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="44" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="22" customHeight="1">
+      <x:c r="A1" s="9" t="str">
+        <x:v>cliente</x:v>
+      </x:c>
+      <x:c r="B1" s="10" t="str">
+        <x:v>telefone</x:v>
+      </x:c>
+      <x:c r="C1" s="10" t="str">
+        <x:v>vencimento</x:v>
+      </x:c>
+      <x:c r="D1" s="11" t="str">
+        <x:v>link_pagamento</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="16" t="str">
+        <x:v>Empresa Aurora</x:v>
+      </x:c>
+      <x:c r="B2" s="19" t="str">
+        <x:v>+55 34 99999-0004</x:v>
+      </x:c>
+      <x:c r="C2" s="22" t="n">
+        <x:v>46231</x:v>
+      </x:c>
+      <x:c r="D2" s="16" t="str">
+        <x:v>https://pagamentos.exemplo/fatura-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="A3" s="17" t="str">
+        <x:v>Comercial Horizonte</x:v>
+      </x:c>
+      <x:c r="B3" s="20" t="str">
+        <x:v>+55 34 99999-0005</x:v>
+      </x:c>
+      <x:c r="C3" s="23" t="n">
+        <x:v>46233</x:v>
+      </x:c>
+      <x:c r="D3" s="17" t="str">
+        <x:v>https://pagamentos.exemplo/fatura-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" s="18" t="str">
+        <x:v>Studio Primavera</x:v>
+      </x:c>
+      <x:c r="B4" s="21" t="str">
+        <x:v>+55 34 99999-0006</x:v>
+      </x:c>
+      <x:c r="C4" s="24" t="n">
+        <x:v>46236</x:v>
+      </x:c>
+      <x:c r="D4" s="18" t="str">
+        <x:v>https://pagamentos.exemplo/fatura-003</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>